<commit_message>
Update PET scoring scripts and supporting files
</commit_message>
<xml_diff>
--- a/PET_Results_Template.xlsx
+++ b/PET_Results_Template.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29721"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kghp.sharepoint.com/sites/RadcomFiles/Shared Documents/General/PET Python Scripts/"/>
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,22 +44,28 @@
     <t>Hot Cell SUVs</t>
   </si>
   <si>
+    <t>Count Rate Performance</t>
+  </si>
+  <si>
     <t>Slice Averages</t>
   </si>
   <si>
+    <t>Max Values</t>
+  </si>
+  <si>
+    <t>Average:</t>
+  </si>
+  <si>
     <t>Average</t>
   </si>
   <si>
+    <t>Result:</t>
+  </si>
+  <si>
     <t>Result</t>
   </si>
   <si>
-    <t>Average:</t>
-  </si>
-  <si>
-    <t>Result:</t>
-  </si>
-  <si>
-    <t>Max Values</t>
+    <t>Min</t>
   </si>
   <si>
     <t>Bone</t>
@@ -69,12 +75,6 @@
   </si>
   <si>
     <t>Water</t>
-  </si>
-  <si>
-    <t>Min</t>
-  </si>
-  <si>
-    <t>Count Rate Performance</t>
   </si>
   <si>
     <t>Images</t>
@@ -90,7 +90,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -146,21 +146,21 @@
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,64 +511,64 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A637B945-5E3E-401C-BC38-4509B1ABD720}">
   <dimension ref="B1:L37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="2:12">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="F1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="J1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-    </row>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="J1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1"/>
-      <c r="J3" s="4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="4"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+    </row>
+    <row r="2" spans="2:12">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+    </row>
+    <row r="3" spans="2:12">
+      <c r="B3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="4"/>
+      <c r="J3" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12">
+      <c r="B4" s="6"/>
       <c r="F4">
         <v>25</v>
       </c>
-      <c r="J4" s="4"/>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="4"/>
+      <c r="J4" s="6"/>
+    </row>
+    <row r="5" spans="2:12">
+      <c r="B5" s="6"/>
       <c r="F5">
         <v>16</v>
       </c>
-      <c r="J5" s="4"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
+      <c r="J5" s="6"/>
+    </row>
+    <row r="6" spans="2:12">
+      <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C6" t="str">
@@ -578,63 +578,63 @@
       <c r="F6">
         <v>12</v>
       </c>
-      <c r="J6" s="3" t="s">
-        <v>3</v>
+      <c r="J6" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="K6" t="str">
         <f>IFERROR(AVERAGE(K3:K5),"")</f>
         <v/>
       </c>
     </row>
-    <row r="7" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="6" t="str">
+    <row r="7" spans="2:12" ht="15.75">
+      <c r="B7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="2" t="str">
         <f>IFERROR(IF(ABS(1-C6)&gt;0.1,"Fail","Pass"),"")</f>
         <v/>
       </c>
       <c r="F7">
         <v>8</v>
       </c>
-      <c r="J7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K7" s="6" t="str">
+      <c r="J7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7" s="2" t="str">
         <f>IFERROR(IF((1-ABS(K6/C6))&gt;0.1,"Pass","Fail"),"")</f>
         <v/>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12">
       <c r="G8" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12">
+      <c r="F9" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12">
+      <c r="F10" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="F9" s="3" t="s">
+    <row r="11" spans="2:12">
+      <c r="F11" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" ht="15.75">
+      <c r="F13" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="F10" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="F11" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="F13" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G13" s="6"/>
-    </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="G13" s="2"/>
+    </row>
+    <row r="15" spans="2:12">
       <c r="B15" s="5" t="s">
         <v>13</v>
       </c>
@@ -649,7 +649,7 @@
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12">
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -662,189 +662,195 @@
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-    </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-    </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-    </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B25" s="2" t="s">
+    <row r="18" spans="2:12">
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+    </row>
+    <row r="19" spans="2:12">
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+    </row>
+    <row r="20" spans="2:12">
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+    </row>
+    <row r="21" spans="2:12">
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+    </row>
+    <row r="22" spans="2:12">
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+    </row>
+    <row r="23" spans="2:12">
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+    </row>
+    <row r="24" spans="2:12">
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+    </row>
+    <row r="25" spans="2:12">
+      <c r="B25" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="F25" s="2" t="s">
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="F25" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="J25" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-    </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-    </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-    </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-    </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-    </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1"/>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="1"/>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B36" s="2" t="s">
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="J25" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+    </row>
+    <row r="26" spans="2:12">
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+    </row>
+    <row r="29" spans="2:12">
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+    </row>
+    <row r="30" spans="2:12">
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+    </row>
+    <row r="31" spans="2:12">
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+    </row>
+    <row r="32" spans="2:12">
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+    </row>
+    <row r="33" spans="2:8">
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+    </row>
+    <row r="34" spans="2:8">
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+    </row>
+    <row r="35" spans="2:8">
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
+    </row>
+    <row r="36" spans="2:8">
+      <c r="B36" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="F36" s="2" t="s">
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="F36" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+    </row>
+    <row r="37" spans="2:8">
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="F1:H2"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="J1:L2"/>
+    <mergeCell ref="J3:J5"/>
     <mergeCell ref="B36:D37"/>
     <mergeCell ref="F29:H35"/>
     <mergeCell ref="F36:H37"/>
@@ -856,12 +862,6 @@
     <mergeCell ref="F25:H26"/>
     <mergeCell ref="J25:L26"/>
     <mergeCell ref="B29:D35"/>
-    <mergeCell ref="B1:D2"/>
-    <mergeCell ref="F1:H2"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="J1:L2"/>
-    <mergeCell ref="J3:J5"/>
   </mergeCells>
   <conditionalFormatting sqref="C7 G13 K7">
     <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Pass">
@@ -876,8 +876,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C6363475C1EEFD49A598447712F3D3E6" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fd4cff7ab8defad676dbfeb75936c5da">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0f805f1a-c809-45d1-8a37-1dbee80eb390" xmlns:ns3="984591a0-cc6c-4327-9f71-f91b2505ea82" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3319200a55eabc991a550a8f2191ae47" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C6363475C1EEFD49A598447712F3D3E6" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="da3fb317689a9f6d13533583b51a848a">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0f805f1a-c809-45d1-8a37-1dbee80eb390" xmlns:ns3="984591a0-cc6c-4327-9f71-f91b2505ea82" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fc47f8e6e5d13c4765c188af9696885d" ns2:_="" ns3:_="">
     <xsd:import namespace="0f805f1a-c809-45d1-8a37-1dbee80eb390"/>
     <xsd:import namespace="984591a0-cc6c-4327-9f71-f91b2505ea82"/>
     <xsd:element name="properties">
@@ -1083,15 +1083,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="984591a0-cc6c-4327-9f71-f91b2505ea82" xsi:nil="true"/>
@@ -1102,14 +1093,23 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4315730-E818-49C0-8F3A-4A626BBAF4FB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49A5DF34-6272-46E7-981D-F51D4C09E8F2}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F72930-DCBF-4B46-A76F-016628EDD0B0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{823AB35B-2678-49B3-88E9-0ED94A22C558}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{823AB35B-2678-49B3-88E9-0ED94A22C558}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F72930-DCBF-4B46-A76F-016628EDD0B0}"/>
 </file>
</xml_diff>